<commit_message>
Final verified pipeline and manuscript-ready code
</commit_message>
<xml_diff>
--- a/reports/tables/Comparison_Full_vs_FirstVisit.xlsx
+++ b/reports/tables/Comparison_Full_vs_FirstVisit.xlsx
@@ -487,12 +487,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.0800</t>
+          <t>0.0729</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.0643</t>
+          <t>0.0745</t>
         </is>
       </c>
     </row>
@@ -504,12 +504,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.0440</t>
+          <t>0.0341</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.0579</t>
+          <t>0.0417</t>
         </is>
       </c>
     </row>
@@ -521,12 +521,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.6831 (0.6091–0.7526)</t>
+          <t>0.6803 (0.6064–0.7535)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.590 (0.491–0.676)</t>
+          <t>0.647 (0.570–0.721)</t>
         </is>
       </c>
     </row>
@@ -538,12 +538,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.1098 (0.0778–0.179)</t>
+          <t>0.1175 (0.0834–0.1973)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.092 (0.062–0.160)</t>
+          <t>0.105 (0.069–0.183)</t>
         </is>
       </c>
     </row>
@@ -555,12 +555,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.0669 (0.0502–0.0838)</t>
+          <t>0.0679 (0.0511–0.0851)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.070 (0.053–0.088)</t>
+          <t>0.064 (0.048–0.081)</t>
         </is>
       </c>
     </row>
@@ -572,12 +572,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>78.0% (64.4–90.0%)</t>
+          <t>73.2% (58.7–86.7%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>48.8% (34.1–64.3%)</t>
+          <t>58.5% (42.5–75.0%)</t>
         </is>
       </c>
     </row>
@@ -589,12 +589,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>53.8% (48.6–59.2%)</t>
+          <t>55.2% (50.2–60.3%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>67.8% (62.4–72.8%)</t>
+          <t>61.3% (56.3–66.6%)</t>
         </is>
       </c>
     </row>
@@ -606,12 +606,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>97.1% (95.1–98.7%)</t>
+          <t>96.5% (94.4–98.4%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>94.7% (92.6–96.7%)</t>
+          <t>95.3% (92.8–97.4%)</t>
         </is>
       </c>
     </row>
@@ -623,12 +623,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.1% (7.8–14.6%)</t>
+          <t>10.8% (7.5–14.5%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10.1% (6.1–14.5%)</t>
+          <t>10.0% (6.4–14.1%)</t>
         </is>
       </c>
     </row>
@@ -640,12 +640,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TP=32 / FP=257 / TN=299 / FN=9</t>
+          <t>TP=30 / FP=249 / TN=307 / FN=11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TP=20 / FP=179 / TN=377 / FN=21</t>
+          <t>TP=24 / FP=215 / TN=341 / FN=17</t>
         </is>
       </c>
     </row>
@@ -657,12 +657,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2.9% (n=306)</t>
+          <t>3.5% (n=318)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.3% (n=396)</t>
+          <t>3.4% (n=296)</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.0% (n=291)</t>
+          <t>10.8% (n=279)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>10.0% (n=201)</t>
+          <t>10.3% (n=301)</t>
         </is>
       </c>
     </row>

</xml_diff>